<commit_message>
chore: 원장 엑셀 갱신 (xlsx → xls 교체) + 0728 PDF 정보 캡처
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ledger_excel/028875_2514.xlsx
+++ b/docs/ledger_excel/028875_2514.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10910"/>
-  <workbookPr defaultThemeVersion="166925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/unanimous0/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\고은환 공유폴더\오늘\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{21268219-04B8-2845-B75C-CEED43C40CA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2F307056-758A-4400-98E3-CC2E7774DEE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3520" yWindow="2660" windowWidth="27900" windowHeight="16940" xr2:uid="{1AB3B13C-DD5B-1E41-91F0-4A089CCEE52C}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{D37ED49C-842B-424A-9C55-5DE99FB2D026}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,52 +36,138 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
-  <si>
-    <t>종목코드</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="30">
+  <si>
+    <t>종목</t>
   </si>
   <si>
     <t>종목명</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>매매구분</t>
   </si>
   <si>
     <t>수량</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>A1167000</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>A5067000</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>삼성전자 F 2607</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>SK하이닉스 F 2607</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>가격</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>금액</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>평균단가</t>
+  </si>
+  <si>
+    <t>현재가</t>
+  </si>
+  <si>
+    <t>평가금액</t>
+  </si>
+  <si>
+    <t>평가손익</t>
+  </si>
+  <si>
+    <t>수수료</t>
+  </si>
+  <si>
+    <t>순손익</t>
+  </si>
+  <si>
+    <t>1GNW4000</t>
+  </si>
+  <si>
+    <t>금양       F 202504 (  10)</t>
+  </si>
+  <si>
+    <t>매수</t>
+  </si>
+  <si>
+    <t>A1168000</t>
+  </si>
+  <si>
+    <t>삼성전자   F 202608 (  10)</t>
+  </si>
+  <si>
+    <t>매도</t>
+  </si>
+  <si>
+    <t>A1A67000</t>
+  </si>
+  <si>
+    <t>한일시멘트 F 202607 (  10)</t>
+  </si>
+  <si>
+    <t>A1B67000</t>
+  </si>
+  <si>
+    <t>HPSP       F 202607 (  10)</t>
+  </si>
+  <si>
+    <t>A5068000</t>
+  </si>
+  <si>
+    <t>SK하이닉스 F 202608 (  10)</t>
+  </si>
+  <si>
+    <t>ACB68000</t>
+  </si>
+  <si>
+    <t>한화솔루션 F 202608 (  10)*</t>
+  </si>
+  <si>
+    <t>AFB67000</t>
+  </si>
+  <si>
+    <t>SK아이이테 F 202607 (  10)</t>
+  </si>
+  <si>
+    <t>AGP67000</t>
+  </si>
+  <si>
+    <t>금호타이어 F 202607 (  10)</t>
+  </si>
+  <si>
+    <t>AHR67000</t>
+  </si>
+  <si>
+    <t>주성엔지니 F 202607 (  10)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
+      <sz val="10"/>
       <color theme="1"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF4D4D4D"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF333333"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFEE595E"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF2375FA"/>
       <name val="맑은 고딕"/>
       <family val="2"/>
       <charset val="129"/>
@@ -117,11 +203,32 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -152,39 +259,39 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546A"/>
+        <a:srgbClr val="0E2841"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
+        <a:srgbClr val="E8E8E8"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="156082"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ED7D31"/>
+        <a:srgbClr val="E97132"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
+        <a:srgbClr val="196B24"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="FFC000"/>
+        <a:srgbClr val="0F9ED5"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="A02B93"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70AD47"/>
+        <a:srgbClr val="4EA72E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563C1"/>
+        <a:srgbClr val="467886"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954F72"/>
+        <a:srgbClr val="96607D"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -236,7 +343,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -347,13 +454,6 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
@@ -362,6 +462,13 @@
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -426,81 +533,363 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC6E6562-DB35-864F-A74B-5ED97E933733}">
-  <dimension ref="A1:E3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
-  <cols>
-    <col min="2" max="2" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13" bestFit="1" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9228D196-7111-4D05-A82A-1C3999810DC4}">
+  <dimension ref="A1:J10"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="1">
-        <v>3000</v>
-      </c>
-      <c r="D2" s="1">
-        <v>295354</v>
-      </c>
-      <c r="E2" s="1">
-        <f>C2*D2</f>
-        <v>886062000</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="1">
-        <v>2000</v>
-      </c>
-      <c r="D3" s="1">
-        <v>1596843</v>
-      </c>
-      <c r="E3" s="1">
-        <f>C3*D3</f>
-        <v>3193686000</v>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="5">
+        <v>4156</v>
+      </c>
+      <c r="E2" s="5">
+        <v>11156</v>
+      </c>
+      <c r="F2" s="5">
+        <v>10720</v>
+      </c>
+      <c r="G2" s="5">
+        <v>445523200</v>
+      </c>
+      <c r="H2" s="6">
+        <v>-18125684</v>
+      </c>
+      <c r="I2" s="3">
+        <v>0</v>
+      </c>
+      <c r="J2" s="6">
+        <v>-18125684</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" s="3">
+        <v>625</v>
+      </c>
+      <c r="E3" s="5">
+        <v>298312</v>
+      </c>
+      <c r="F3" s="5">
+        <v>271500</v>
+      </c>
+      <c r="G3" s="5">
+        <v>1696875000</v>
+      </c>
+      <c r="H3" s="8">
+        <v>167575000</v>
+      </c>
+      <c r="I3" s="3">
+        <v>0</v>
+      </c>
+      <c r="J3" s="8">
+        <v>167575000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="3">
+        <v>21</v>
+      </c>
+      <c r="E4" s="5">
+        <v>13613</v>
+      </c>
+      <c r="F4" s="5">
+        <v>14240</v>
+      </c>
+      <c r="G4" s="5">
+        <v>2990400</v>
+      </c>
+      <c r="H4" s="8">
+        <v>131607</v>
+      </c>
+      <c r="I4" s="3">
+        <v>0</v>
+      </c>
+      <c r="J4" s="8">
+        <v>131607</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="3">
+        <v>256</v>
+      </c>
+      <c r="E5" s="5">
+        <v>51822</v>
+      </c>
+      <c r="F5" s="5">
+        <v>38600</v>
+      </c>
+      <c r="G5" s="5">
+        <v>98816000</v>
+      </c>
+      <c r="H5" s="6">
+        <v>-33848980</v>
+      </c>
+      <c r="I5" s="3">
+        <v>0</v>
+      </c>
+      <c r="J5" s="6">
+        <v>-33848980</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="5">
+        <v>7941</v>
+      </c>
+      <c r="E6" s="5">
+        <v>2343157</v>
+      </c>
+      <c r="F6" s="5">
+        <v>2120000</v>
+      </c>
+      <c r="G6" s="5">
+        <v>168349200000</v>
+      </c>
+      <c r="H6" s="8">
+        <v>17720930000</v>
+      </c>
+      <c r="I6" s="3">
+        <v>0</v>
+      </c>
+      <c r="J6" s="8">
+        <v>17720930000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="3">
+        <v>485</v>
+      </c>
+      <c r="E7" s="5">
+        <v>30156</v>
+      </c>
+      <c r="F7" s="5">
+        <v>29750</v>
+      </c>
+      <c r="G7" s="5">
+        <v>153058581</v>
+      </c>
+      <c r="H7" s="6">
+        <v>-2090284</v>
+      </c>
+      <c r="I7" s="3">
+        <v>0</v>
+      </c>
+      <c r="J7" s="6">
+        <v>-2090284</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="3">
+        <v>349</v>
+      </c>
+      <c r="E8" s="5">
+        <v>16440</v>
+      </c>
+      <c r="F8" s="5">
+        <v>14260</v>
+      </c>
+      <c r="G8" s="5">
+        <v>49767400</v>
+      </c>
+      <c r="H8" s="6">
+        <v>-7609072</v>
+      </c>
+      <c r="I8" s="3">
+        <v>0</v>
+      </c>
+      <c r="J8" s="6">
+        <v>-7609072</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" s="3">
+        <v>154</v>
+      </c>
+      <c r="E9" s="5">
+        <v>4957</v>
+      </c>
+      <c r="F9" s="5">
+        <v>5440</v>
+      </c>
+      <c r="G9" s="5">
+        <v>8377600</v>
+      </c>
+      <c r="H9" s="8">
+        <v>743300</v>
+      </c>
+      <c r="I9" s="3">
+        <v>0</v>
+      </c>
+      <c r="J9" s="8">
+        <v>743300</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" s="3">
+        <v>139</v>
+      </c>
+      <c r="E10" s="5">
+        <v>218081</v>
+      </c>
+      <c r="F10" s="5">
+        <v>161200</v>
+      </c>
+      <c r="G10" s="5">
+        <v>224068000</v>
+      </c>
+      <c r="H10" s="6">
+        <v>-79065000</v>
+      </c>
+      <c r="I10" s="3">
+        <v>0</v>
+      </c>
+      <c r="J10" s="6">
+        <v>-79065000</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>